<commit_message>
Add Enterprise Custom HTML Reporter and update metadata handling
</commit_message>
<xml_diff>
--- a/data/testRegistry.xlsx
+++ b/data/testRegistry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manishgangwar/LearnPlaywright/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8541BD3F-8B34-1247-8293-621C933BAFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5EA5B1F-BD68-3B4E-B82F-9878B7E6D6DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10520" yWindow="1780" windowWidth="28040" windowHeight="17180" activeTab="3" xr2:uid="{20BDFCB9-813F-5B44-AE4E-B81527177D88}"/>
+    <workbookView xWindow="10360" yWindow="1780" windowWidth="28040" windowHeight="17180" xr2:uid="{20BDFCB9-813F-5B44-AE4E-B81527177D88}"/>
   </bookViews>
   <sheets>
     <sheet name="Registry" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="40">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>webkit</t>
+  </si>
+  <si>
+    <t>@smoke, @critical</t>
   </si>
 </sst>
 </file>
@@ -621,7 +624,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
@@ -630,7 +633,7 @@
         <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
feat: enhance security, improve performance, and update HTTP reports
</commit_message>
<xml_diff>
--- a/data/testRegistry.xlsx
+++ b/data/testRegistry.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manishgangwar/LearnPlaywright/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5EA5B1F-BD68-3B4E-B82F-9878B7E6D6DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180EE30E-CDEB-134F-932C-5C090497648B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10360" yWindow="1780" windowWidth="28040" windowHeight="17180" xr2:uid="{20BDFCB9-813F-5B44-AE4E-B81527177D88}"/>
+    <workbookView xWindow="10360" yWindow="1780" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{20BDFCB9-813F-5B44-AE4E-B81527177D88}"/>
   </bookViews>
   <sheets>
-    <sheet name="Registry" sheetId="1" r:id="rId1"/>
-    <sheet name="Login" sheetId="2" r:id="rId2"/>
-    <sheet name="ProductPage" sheetId="3" r:id="rId3"/>
-    <sheet name="Cart" sheetId="4" r:id="rId4"/>
+    <sheet name="Metadata" sheetId="5" r:id="rId1"/>
+    <sheet name="Registry" sheetId="1" r:id="rId2"/>
+    <sheet name="Login" sheetId="2" r:id="rId3"/>
+    <sheet name="ProductPage" sheetId="3" r:id="rId4"/>
+    <sheet name="Cart" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="46">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -159,13 +160,31 @@
   </si>
   <si>
     <t>@smoke, @critical</t>
+  </si>
+  <si>
+    <t>chrome</t>
+  </si>
+  <si>
+    <t>chromium</t>
+  </si>
+  <si>
+    <t>edge</t>
+  </si>
+  <si>
+    <t>@smoke</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>P3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -184,6 +203,13 @@
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -207,10 +233,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -544,6 +571,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{432BEF4D-2BCF-854A-AEE7-E4BA21F2B677}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A1F7C2-3FA6-A04B-8A49-A93E4A58F39F}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -555,7 +627,7 @@
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19" x14ac:dyDescent="0.25">
@@ -607,7 +679,7 @@
         <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -633,7 +705,7 @@
         <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -647,10 +719,10 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
         <v>12</v>
@@ -659,12 +731,12 @@
         <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
@@ -673,7 +745,7 @@
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>11</v>
@@ -689,12 +761,25 @@
       </c>
     </row>
   </sheetData>
+  <dataConsolidate/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{602F1445-31BC-8545-A5AD-E5669BF1D977}">
+          <x14:formula1>
+            <xm:f>Metadata!$A$2:$A$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F283B292-7C67-804C-B2DD-7E931E27676D}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -747,7 +832,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C91DC712-EAB6-2641-98BD-30F2E7CCF035}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -824,7 +909,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B885C31-9163-7B4B-BF19-F80883ACC645}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>